<commit_message>
Clear check-in status from demo template and optimize mobile-responsive layouts for scanner and dashboard pages
</commit_message>
<xml_diff>
--- a/data_with_qrdemo.xlsx
+++ b/data_with_qrdemo.xlsx
@@ -937,11 +937,6 @@
 ID: 0L1EB1GO</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Scanned 3 Times</t>
-        </is>
-      </c>
     </row>
     <row r="3" ht="75" customHeight="1">
       <c r="A3" t="inlineStr">
@@ -970,11 +965,6 @@
 Email: jane@example.com
 Reg No: REG002
 ID: 19E8AX9P</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Scanned</t>
         </is>
       </c>
     </row>

</xml_diff>